<commit_message>
Remove unnecessary Zone.Identifier file and add modified Excel files for Zive data analysis.
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/06_Anotacijos_logai/06.1_Anotavimo_logas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/06_Anotacijos_logai/06.1_Anotavimo_logas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AnotacijosLogai\06_Anotacijos_logai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F085E71D-59A1-4A1E-9452-0FFFCD3FE61A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E8147C-24CF-423D-B2DD-120F42D01289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="86">
   <si>
     <t>filename</t>
   </si>
@@ -290,6 +290,12 @@
   </si>
   <si>
     <t xml:space="preserve">Labai geras </t>
+  </si>
+  <si>
+    <t>2222, neatnaujintas lokaliai</t>
+  </si>
+  <si>
+    <t>1111, neatnaujintas lokaliai</t>
   </si>
 </sst>
 </file>
@@ -1570,10 +1576,9 @@
       <c r="G2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H2" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J2" s="5"/>
       <c r="K2" s="8"/>
       <c r="L2" t="s">
@@ -1582,6 +1587,9 @@
       <c r="M2" t="s">
         <v>24</v>
       </c>
+      <c r="N2" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
@@ -1603,10 +1611,9 @@
       <c r="G3" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J3" s="5"/>
       <c r="K3" s="8"/>
       <c r="L3" t="s">
@@ -1615,9 +1622,8 @@
       <c r="M3" t="s">
         <v>29</v>
       </c>
-      <c r="N3" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N3" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.35">
@@ -1640,10 +1646,9 @@
       <c r="G4" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="5"/>
+      <c r="I4" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J4" s="5"/>
       <c r="K4" s="8"/>
       <c r="L4" t="s">
@@ -1652,9 +1657,8 @@
       <c r="M4" t="s">
         <v>29</v>
       </c>
-      <c r="N4" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
@@ -1677,10 +1681,10 @@
       <c r="G5" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J5" s="5"/>
       <c r="K5" s="8"/>
       <c r="L5" t="s">
@@ -1689,9 +1693,8 @@
       <c r="M5" t="s">
         <v>36</v>
       </c>
-      <c r="N5" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
@@ -1714,10 +1717,9 @@
       <c r="G6" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="5"/>
+      <c r="I6" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J6" s="5"/>
       <c r="K6" s="8"/>
       <c r="L6" t="s">
@@ -1726,9 +1728,8 @@
       <c r="M6" t="s">
         <v>38</v>
       </c>
-      <c r="N6" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N6" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
@@ -1751,10 +1752,9 @@
       <c r="G7" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="5"/>
+      <c r="I7" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J7" s="5"/>
       <c r="K7" s="8"/>
       <c r="L7" t="s">
@@ -1763,9 +1763,8 @@
       <c r="M7" t="s">
         <v>41</v>
       </c>
-      <c r="N7" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N7" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">
@@ -1788,10 +1787,9 @@
       <c r="G8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" s="5"/>
+      <c r="I8" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J8" s="5"/>
       <c r="K8" s="8"/>
       <c r="L8" t="s">
@@ -1800,9 +1798,8 @@
       <c r="M8" t="s">
         <v>45</v>
       </c>
-      <c r="N8" t="str">
-        <f>""</f>
-        <v/>
+      <c r="N8" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.35">
@@ -1822,12 +1819,14 @@
       <c r="G9" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="5"/>
+      <c r="I9" s="5" t="b">
+        <v>1</v>
+      </c>
       <c r="J9" s="5"/>
       <c r="K9" s="8"/>
+      <c r="N9" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>

</xml_diff>